<commit_message>
Recompute matching analysis with threshold 0.5
</commit_message>
<xml_diff>
--- a/analysis(S4)/tables/level3_agent_topic_matching_analysis.xlsx
+++ b/analysis(S4)/tables/level3_agent_topic_matching_analysis.xlsx
@@ -758,10 +758,10 @@
         <v>1142</v>
       </c>
       <c r="C4">
-        <v>0.5979711570167997</v>
+        <v>0.4893840372786735</v>
       </c>
       <c r="D4">
-        <v>0.4386570565625684</v>
+        <v>0.4610758805254378</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -770,10 +770,10 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>0.06732673267326733</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="I4">
         <v>1</v>
@@ -1415,19 +1415,19 @@
         <v>75</v>
       </c>
       <c r="E15">
-        <v>3.768747692276521</v>
+        <v>4.248478831706663</v>
       </c>
       <c r="F15">
-        <v>9.858411101812312</v>
+        <v>10.83982054634164</v>
       </c>
       <c r="G15">
-        <v>0.7022480984782935</v>
+        <v>0.6951080296905583</v>
       </c>
       <c r="H15">
-        <v>-15.55338301206544</v>
+        <v>-16.99717903800025</v>
       </c>
       <c r="I15">
-        <v>23.09087839661848</v>
+        <v>25.49413670141358</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -1444,19 +1444,19 @@
         <v>80</v>
       </c>
       <c r="E16">
-        <v>2.331458857690044</v>
+        <v>2.243837435745824</v>
       </c>
       <c r="F16">
-        <v>3.353882984654907</v>
+        <v>2.524100167109841</v>
       </c>
       <c r="G16">
-        <v>0.4869599763134116</v>
+        <v>0.3740217346552139</v>
       </c>
       <c r="H16">
-        <v>-4.242031000595276</v>
+        <v>-2.703307985160997</v>
       </c>
       <c r="I16">
-        <v>8.904948715975364</v>
+        <v>7.190982856652644</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -1473,19 +1473,19 @@
         <v>81</v>
       </c>
       <c r="E17">
-        <v>0.9012070061595064</v>
+        <v>0.8138195382517793</v>
       </c>
       <c r="F17">
-        <v>9.851251400021214</v>
+        <v>10.82807355074326</v>
       </c>
       <c r="G17">
-        <v>0.9271100255189695</v>
+        <v>0.9400887668133382</v>
       </c>
       <c r="H17">
-        <v>-18.40689094053186</v>
+        <v>-20.40881464315576</v>
       </c>
       <c r="I17">
-        <v>20.20930495285087</v>
+        <v>22.03645371965931</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -1502,19 +1502,19 @@
         <v>82</v>
       </c>
       <c r="E18">
-        <v>-1.960476632684216</v>
+        <v>-3.155046630895897</v>
       </c>
       <c r="F18">
-        <v>9.964722762465048</v>
+        <v>21.6145318460818</v>
       </c>
       <c r="G18">
-        <v>0.8440296652031867</v>
+        <v>0.8839460421363635</v>
       </c>
       <c r="H18">
-        <v>-21.49097436304218</v>
+        <v>-45.51875059191028</v>
       </c>
       <c r="I18">
-        <v>17.57002109767375</v>
+        <v>39.20865733011848</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -1531,19 +1531,19 @@
         <v>83</v>
       </c>
       <c r="E19">
-        <v>-0.4177201246240076</v>
+        <v>-0.3296787474704433</v>
       </c>
       <c r="F19">
-        <v>9.847845891115433</v>
+        <v>10.82468101015505</v>
       </c>
       <c r="G19">
-        <v>0.9661659490316031</v>
+        <v>0.9757032173010241</v>
       </c>
       <c r="H19">
-        <v>-19.71914339651101</v>
+        <v>-21.54566367150899</v>
       </c>
       <c r="I19">
-        <v>18.883703147263</v>
+        <v>20.88630617656811</v>
       </c>
     </row>
     <row r="20" spans="1:10">
@@ -1560,19 +1560,19 @@
         <v>84</v>
       </c>
       <c r="E20">
-        <v>-0.1937700263819698</v>
+        <v>-0.116995911111562</v>
       </c>
       <c r="F20">
-        <v>9.849491725450276</v>
+        <v>10.82598899805447</v>
       </c>
       <c r="G20">
-        <v>0.9843041504682478</v>
+        <v>0.9913774700716474</v>
       </c>
       <c r="H20">
-        <v>-19.49841907428979</v>
+        <v>-21.33554444432519</v>
       </c>
       <c r="I20">
-        <v>19.11087902152585</v>
+        <v>21.10155262210206</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -1589,19 +1589,19 @@
         <v>85</v>
       </c>
       <c r="E21">
-        <v>-0.1520868063505111</v>
+        <v>-0.1361299221374689</v>
       </c>
       <c r="F21">
-        <v>0.1376814687988474</v>
+        <v>0.1337216547395195</v>
       </c>
       <c r="G21">
-        <v>0.2693208106335139</v>
+        <v>0.3086734156099772</v>
       </c>
       <c r="H21">
-        <v>-0.4219375265348271</v>
+        <v>-0.398219549380027</v>
       </c>
       <c r="I21">
-        <v>0.1177639138338049</v>
+        <v>0.1259597051050891</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -1618,22 +1618,22 @@
         <v>92</v>
       </c>
       <c r="E22">
-        <v>0.9376467025568098</v>
+        <v>1.546515885165592</v>
       </c>
       <c r="F22">
-        <v>0.3683721372607643</v>
+        <v>0.5499977861978362</v>
       </c>
       <c r="G22">
-        <v>0.01091591880427608</v>
+        <v>0.004925618471828861</v>
       </c>
       <c r="H22">
-        <v>0.2156505806176664</v>
+        <v>0.4685400326410722</v>
       </c>
       <c r="I22">
-        <v>1.659642824495953</v>
+        <v>2.624491737690112</v>
       </c>
       <c r="J22">
-        <v>0.9376467025568098</v>
+        <v>1.546515885165592</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -1650,22 +1650,22 @@
         <v>87</v>
       </c>
       <c r="E23">
-        <v>0.2039561605882623</v>
+        <v>0.1442727583266606</v>
       </c>
       <c r="F23">
-        <v>0.1108020597310869</v>
+        <v>0.1021174793657897</v>
       </c>
       <c r="G23">
-        <v>0.0656618165557489</v>
+        <v>0.157711129716964</v>
       </c>
       <c r="H23">
-        <v>-0.0132118858975239</v>
+        <v>-0.05587382342229941</v>
       </c>
       <c r="I23">
-        <v>0.4211242070740485</v>
+        <v>0.3444193400756206</v>
       </c>
       <c r="J23">
-        <v>0.2039561605882623</v>
+        <v>0.1442727583266606</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -1682,22 +1682,22 @@
         <v>88</v>
       </c>
       <c r="E24">
-        <v>0.007212615504369017</v>
+        <v>0.05084352044059733</v>
       </c>
       <c r="F24">
-        <v>0.2526590322802555</v>
+        <v>0.2491638513080231</v>
       </c>
       <c r="G24">
-        <v>0.9772260149409779</v>
+        <v>0.8383092936623524</v>
       </c>
       <c r="H24">
-        <v>-0.4879899881336748</v>
+        <v>-0.4375086543724213</v>
       </c>
       <c r="I24">
-        <v>0.5024152191424128</v>
+        <v>0.5391956952536159</v>
       </c>
       <c r="J24">
-        <v>0.007212615504369017</v>
+        <v>0.05084352044059733</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -1714,22 +1714,22 @@
         <v>89</v>
       </c>
       <c r="E25">
-        <v>-1.084539152377894</v>
+        <v>-1.056605498875292</v>
       </c>
       <c r="F25">
-        <v>0.4095347608645611</v>
+        <v>0.4030533154527287</v>
       </c>
       <c r="G25">
-        <v>0.008091625911413106</v>
+        <v>0.008754297701142593</v>
       </c>
       <c r="H25">
-        <v>-1.887212534089657</v>
+        <v>-1.846575481012102</v>
       </c>
       <c r="I25">
-        <v>-0.2818657706661304</v>
+        <v>-0.2666355167384827</v>
       </c>
       <c r="J25">
-        <v>-1.084539152377894</v>
+        <v>-1.056605498875292</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -1746,22 +1746,22 @@
         <v>90</v>
       </c>
       <c r="E26">
-        <v>0.7812553935753863</v>
+        <v>0.7333888968278429</v>
       </c>
       <c r="F26">
-        <v>0.3077800323877884</v>
+        <v>0.3102800945842114</v>
       </c>
       <c r="G26">
-        <v>0.01113745213170189</v>
+        <v>0.01809663115522448</v>
       </c>
       <c r="H26">
-        <v>0.1780176149347495</v>
+        <v>0.1252510863231072</v>
       </c>
       <c r="I26">
-        <v>1.384493172216023</v>
+        <v>1.341526707332579</v>
       </c>
       <c r="J26">
-        <v>0.7812553935753863</v>
+        <v>0.7333888968278429</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -1778,22 +1778,22 @@
         <v>91</v>
       </c>
       <c r="E27">
-        <v>0.09042056682961208</v>
+        <v>0.06751518199563347</v>
       </c>
       <c r="F27">
-        <v>0.2141185223125586</v>
+        <v>0.2074492045303057</v>
       </c>
       <c r="G27">
-        <v>0.6728118019428135</v>
+        <v>0.7448374605320107</v>
       </c>
       <c r="H27">
-        <v>-0.3292440253259387</v>
+        <v>-0.3390777875052492</v>
       </c>
       <c r="I27">
-        <v>0.5100851589851628</v>
+        <v>0.4741081514965162</v>
       </c>
       <c r="J27">
-        <v>0.09042056682961208</v>
+        <v>0.06751518199563347</v>
       </c>
     </row>
   </sheetData>
@@ -1967,7 +1967,7 @@
         <v>0.2521920282351128</v>
       </c>
       <c r="F6">
-        <v>0.1554940311481034</v>
+        <v>0.05011315680343081</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2027,7 +2027,7 @@
         <v>0.6564982279693488</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>0.7816666666666666</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2087,7 +2087,7 @@
         <v>0.5065151515151516</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>0.8787878787878788</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2127,7 +2127,7 @@
         <v>0.3696966914246096</v>
       </c>
       <c r="F14">
-        <v>0.4185958656407259</v>
+        <v>0.1968117890127723</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2147,7 +2147,7 @@
         <v>0.28955</v>
       </c>
       <c r="F15">
-        <v>0.1666666666666667</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2167,7 +2167,7 @@
         <v>0.2440803931451613</v>
       </c>
       <c r="F16">
-        <v>0.046875</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -2247,7 +2247,7 @@
         <v>0.3195803291787255</v>
       </c>
       <c r="F20">
-        <v>0.1985614243281433</v>
+        <v>0.07496900346120439</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2267,7 +2267,7 @@
         <v>0.3059375</v>
       </c>
       <c r="F21">
-        <v>0.2013888888888889</v>
+        <v>0.09722222222222222</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -2337,10 +2337,10 @@
         <v>46</v>
       </c>
       <c r="D2">
-        <v>6.327057380804667</v>
+        <v>5.274472723445769</v>
       </c>
       <c r="E2">
-        <v>0.8634957781872872</v>
+        <v>0.917698495030173</v>
       </c>
       <c r="F2" t="s">
         <v>47</v>
@@ -2454,13 +2454,13 @@
         <v>1142</v>
       </c>
       <c r="E4">
-        <v>3457.243155065492</v>
+        <v>3455.3712488721</v>
       </c>
       <c r="F4">
-        <v>3542.932273699163</v>
+        <v>3541.060367505771</v>
       </c>
       <c r="G4">
-        <v>0.2252068558160921</v>
+        <v>0.2264758156005846</v>
       </c>
       <c r="I4" t="s">
         <v>66</v>
@@ -2480,13 +2480,13 @@
         <v>1142</v>
       </c>
       <c r="E5">
-        <v>3674.110604186647</v>
+        <v>3673.043584197633</v>
       </c>
       <c r="F5">
-        <v>3759.799722820318</v>
+        <v>3758.732702831304</v>
       </c>
       <c r="G5">
-        <v>0.23027942674959</v>
+        <v>0.230998274092541</v>
       </c>
       <c r="I5" t="s">
         <v>66</v>
@@ -2532,13 +2532,13 @@
         <v>126</v>
       </c>
       <c r="E7">
-        <v>262.4070276459344</v>
+        <v>260.5765054617245</v>
       </c>
       <c r="F7">
-        <v>299.2786924363036</v>
+        <v>297.4481702520937</v>
       </c>
       <c r="G7">
-        <v>0.3002978010149173</v>
+        <v>0.3103895584745069</v>
       </c>
       <c r="I7" t="s">
         <v>66</v>
@@ -3652,19 +3652,19 @@
         <v>75</v>
       </c>
       <c r="E36">
-        <v>2.673580446244357</v>
+        <v>2.650831443769448</v>
       </c>
       <c r="F36">
-        <v>0.6538428187428393</v>
+        <v>0.6193963735871511</v>
       </c>
       <c r="G36">
-        <v>4.331878429922007E-05</v>
+        <v>1.871443363163149E-05</v>
       </c>
       <c r="H36">
-        <v>1.392072069958241</v>
+        <v>1.436836859383915</v>
       </c>
       <c r="I36">
-        <v>3.955088822530473</v>
+        <v>3.86482602815498</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -3681,19 +3681,19 @@
         <v>76</v>
       </c>
       <c r="E37">
-        <v>-0.4759116701517649</v>
+        <v>-0.4368736338364723</v>
       </c>
       <c r="F37">
-        <v>0.6150640742251555</v>
+        <v>0.6150627017365585</v>
       </c>
       <c r="G37">
-        <v>0.439073027083338</v>
+        <v>0.4775235663192308</v>
       </c>
       <c r="H37">
-        <v>-1.68141510381754</v>
+        <v>-1.642374377474028</v>
       </c>
       <c r="I37">
-        <v>0.7295917635140103</v>
+        <v>0.7686271098010837</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -3710,19 +3710,19 @@
         <v>77</v>
       </c>
       <c r="E38">
-        <v>0.1873998697763583</v>
+        <v>0.2005722947968448</v>
       </c>
       <c r="F38">
-        <v>0.4780886936447536</v>
+        <v>0.4749307718727442</v>
       </c>
       <c r="G38">
-        <v>0.6950750567419234</v>
+        <v>0.6727921822234209</v>
       </c>
       <c r="H38">
-        <v>-0.7496367511831623</v>
+        <v>-0.7302749132235424</v>
       </c>
       <c r="I38">
-        <v>1.124436490735879</v>
+        <v>1.131419502817232</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -3739,19 +3739,19 @@
         <v>78</v>
       </c>
       <c r="E39">
-        <v>-0.5363282820321476</v>
+        <v>-0.458266560036831</v>
       </c>
       <c r="F39">
-        <v>0.4748688485101474</v>
+        <v>0.4738273927997891</v>
       </c>
       <c r="G39">
-        <v>0.2587190064143159</v>
+        <v>0.3334644148491658</v>
       </c>
       <c r="H39">
-        <v>-1.467054122492043</v>
+        <v>-1.386951184812931</v>
       </c>
       <c r="I39">
-        <v>0.3943975584277483</v>
+        <v>0.470418064739269</v>
       </c>
     </row>
     <row r="40" spans="1:10">
@@ -3768,19 +3768,19 @@
         <v>79</v>
       </c>
       <c r="E40">
-        <v>-0.1899365739910334</v>
+        <v>-0.1243473660297038</v>
       </c>
       <c r="F40">
-        <v>0.4995673387581321</v>
+        <v>0.4962191239782717</v>
       </c>
       <c r="G40">
-        <v>0.7037953667821595</v>
+        <v>0.8021314010311725</v>
       </c>
       <c r="H40">
-        <v>-1.169070565809493</v>
+        <v>-1.096918977467132</v>
       </c>
       <c r="I40">
-        <v>0.7891974178274261</v>
+        <v>0.8482242454077247</v>
       </c>
     </row>
     <row r="41" spans="1:10">
@@ -3797,19 +3797,19 @@
         <v>80</v>
       </c>
       <c r="E41">
-        <v>0.9178609037636835</v>
+        <v>0.9753799578724875</v>
       </c>
       <c r="F41">
-        <v>0.5283348184988516</v>
+        <v>0.5279420072609138</v>
       </c>
       <c r="G41">
-        <v>0.08233929930797947</v>
+        <v>0.06467276099463994</v>
       </c>
       <c r="H41">
-        <v>-0.1176563122725719</v>
+        <v>-0.05936736228468709</v>
       </c>
       <c r="I41">
-        <v>1.953378119799939</v>
+        <v>2.010127278029662</v>
       </c>
     </row>
     <row r="42" spans="1:10">
@@ -3826,19 +3826,19 @@
         <v>81</v>
       </c>
       <c r="E42">
-        <v>1.515992368097837</v>
+        <v>1.481236754354238</v>
       </c>
       <c r="F42">
-        <v>0.467162838937492</v>
+        <v>0.423261125683762</v>
       </c>
       <c r="G42">
-        <v>0.001174074085358433</v>
+        <v>0.0004659893382918971</v>
       </c>
       <c r="H42">
-        <v>0.6003700288648666</v>
+        <v>0.6516601919581837</v>
       </c>
       <c r="I42">
-        <v>2.431614707330807</v>
+        <v>2.310813316750293</v>
       </c>
     </row>
     <row r="43" spans="1:10">
@@ -3855,19 +3855,19 @@
         <v>82</v>
       </c>
       <c r="E43">
-        <v>-0.006509875603339267</v>
+        <v>-0.02733033283988958</v>
       </c>
       <c r="F43">
-        <v>0.4608505511379853</v>
+        <v>0.4162870687271246</v>
       </c>
       <c r="G43">
-        <v>0.9887296293961568</v>
+        <v>0.9476544021900747</v>
       </c>
       <c r="H43">
-        <v>-0.9097603580892248</v>
+        <v>-0.8432379947748041</v>
       </c>
       <c r="I43">
-        <v>0.8967406068825463</v>
+        <v>0.7885773290950249</v>
       </c>
     </row>
     <row r="44" spans="1:10">
@@ -3884,19 +3884,19 @@
         <v>83</v>
       </c>
       <c r="E44">
-        <v>0.1270054165199945</v>
+        <v>0.1012275299358363</v>
       </c>
       <c r="F44">
-        <v>0.4557355605229069</v>
+        <v>0.4102966825768818</v>
       </c>
       <c r="G44">
-        <v>0.7804886769118889</v>
+        <v>0.8051265637812437</v>
       </c>
       <c r="H44">
-        <v>-0.766219868579077</v>
+        <v>-0.7029391908911148</v>
       </c>
       <c r="I44">
-        <v>1.020230701619066</v>
+        <v>0.9053942507627873</v>
       </c>
     </row>
     <row r="45" spans="1:10">
@@ -3913,19 +3913,19 @@
         <v>84</v>
       </c>
       <c r="E45">
-        <v>0.2090054432531918</v>
+        <v>0.1746032311309405</v>
       </c>
       <c r="F45">
-        <v>0.464283277309252</v>
+        <v>0.4201311291710433</v>
       </c>
       <c r="G45">
-        <v>0.6525893564332554</v>
+        <v>0.6777084163393503</v>
       </c>
       <c r="H45">
-        <v>-0.7009730588971648</v>
+        <v>-0.6488386508284496</v>
       </c>
       <c r="I45">
-        <v>1.118983945403548</v>
+        <v>0.9980451130903307</v>
       </c>
     </row>
     <row r="46" spans="1:10">
@@ -3942,19 +3942,19 @@
         <v>85</v>
       </c>
       <c r="E46">
-        <v>-0.1441172481474865</v>
+        <v>-0.1444872734477802</v>
       </c>
       <c r="F46">
-        <v>0.0686700094957773</v>
+        <v>0.06840188923815181</v>
       </c>
       <c r="G46">
-        <v>0.03584399794840255</v>
+        <v>0.03465826624998593</v>
       </c>
       <c r="H46">
-        <v>-0.2787079935772335</v>
+        <v>-0.2785525128290557</v>
       </c>
       <c r="I46">
-        <v>-0.009526502717739471</v>
+        <v>-0.01042203406650477</v>
       </c>
     </row>
     <row r="47" spans="1:10">
@@ -3971,22 +3971,22 @@
         <v>92</v>
       </c>
       <c r="E47">
-        <v>0.08507393934414627</v>
+        <v>0.1202663167196417</v>
       </c>
       <c r="F47">
-        <v>0.04279734072696693</v>
+        <v>0.04910708160623352</v>
       </c>
       <c r="G47">
-        <v>0.04683023216695149</v>
+        <v>0.01432285546906641</v>
       </c>
       <c r="H47">
-        <v>0.001192692885201838</v>
+        <v>0.02401820538555463</v>
       </c>
       <c r="I47">
-        <v>0.1689551858030907</v>
+        <v>0.2165144280537287</v>
       </c>
       <c r="J47">
-        <v>0.08507393934414627</v>
+        <v>0.1202663167196417</v>
       </c>
     </row>
     <row r="48" spans="1:10">
@@ -4003,22 +4003,22 @@
         <v>87</v>
       </c>
       <c r="E48">
-        <v>0.2404797137903958</v>
+        <v>0.2332540657343897</v>
       </c>
       <c r="F48">
-        <v>0.03617694442999952</v>
+        <v>0.03357390267961636</v>
       </c>
       <c r="G48">
-        <v>2.98478351955559E-11</v>
+        <v>3.718649685130255E-12</v>
       </c>
       <c r="H48">
-        <v>0.1695742056368899</v>
+        <v>0.1674504256618888</v>
       </c>
       <c r="I48">
-        <v>0.3113852219439018</v>
+        <v>0.2990577058068906</v>
       </c>
       <c r="J48">
-        <v>0.2404797137903958</v>
+        <v>0.2332540657343897</v>
       </c>
     </row>
     <row r="49" spans="1:10">
@@ -4035,22 +4035,22 @@
         <v>88</v>
       </c>
       <c r="E49">
-        <v>0.1010455754263736</v>
+        <v>0.1119334829522838</v>
       </c>
       <c r="F49">
-        <v>0.07297990052432075</v>
+        <v>0.07279088684226569</v>
       </c>
       <c r="G49">
-        <v>0.1661848513096016</v>
+        <v>0.1241121164561368</v>
       </c>
       <c r="H49">
-        <v>-0.04199240119661085</v>
+        <v>-0.03073403366128741</v>
       </c>
       <c r="I49">
-        <v>0.2440835520493581</v>
+        <v>0.2546009995658551</v>
       </c>
       <c r="J49">
-        <v>0.1010455754263736</v>
+        <v>0.1119334829522838</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -4067,22 +4067,22 @@
         <v>89</v>
       </c>
       <c r="E50">
-        <v>-0.2443126750009654</v>
+        <v>-0.2389990920125367</v>
       </c>
       <c r="F50">
-        <v>0.06103421399288912</v>
+        <v>0.06109751606328423</v>
       </c>
       <c r="G50">
-        <v>6.257587024254461E-05</v>
+        <v>9.162424994774614E-05</v>
       </c>
       <c r="H50">
-        <v>-0.3639375362517386</v>
+        <v>-0.3587480230414313</v>
       </c>
       <c r="I50">
-        <v>-0.1246878137501921</v>
+        <v>-0.1192501609836422</v>
       </c>
       <c r="J50">
-        <v>-0.2443126750009654</v>
+        <v>-0.2389990920125367</v>
       </c>
     </row>
     <row r="51" spans="1:10">
@@ -4099,22 +4099,22 @@
         <v>90</v>
       </c>
       <c r="E51">
-        <v>0.1809860219979053</v>
+        <v>0.1840575368527516</v>
       </c>
       <c r="F51">
-        <v>0.06558352767138007</v>
+        <v>0.06476563657966095</v>
       </c>
       <c r="G51">
-        <v>0.005786752972493485</v>
+        <v>0.004484539438764956</v>
       </c>
       <c r="H51">
-        <v>0.05244466978291434</v>
+        <v>0.05711922172080622</v>
       </c>
       <c r="I51">
-        <v>0.3095273742128963</v>
+        <v>0.3109958519846969</v>
       </c>
       <c r="J51">
-        <v>0.1809860219979053</v>
+        <v>0.1840575368527516</v>
       </c>
     </row>
     <row r="52" spans="1:10">
@@ -4131,22 +4131,22 @@
         <v>91</v>
       </c>
       <c r="E52">
-        <v>0.01407222843247241</v>
+        <v>0.01750108683967624</v>
       </c>
       <c r="F52">
-        <v>0.04890712148265239</v>
+        <v>0.04936878554154801</v>
       </c>
       <c r="G52">
-        <v>0.7735505694301237</v>
+        <v>0.7229664447515003</v>
       </c>
       <c r="H52">
-        <v>-0.08178396826105144</v>
+        <v>-0.0792599547822396</v>
       </c>
       <c r="I52">
-        <v>0.1099284251259963</v>
+        <v>0.1142621284615921</v>
       </c>
       <c r="J52">
-        <v>0.01407222843247241</v>
+        <v>0.01750108683967624</v>
       </c>
     </row>
     <row r="53" spans="1:10">
@@ -4163,19 +4163,19 @@
         <v>75</v>
       </c>
       <c r="E53">
-        <v>3.003072517434528</v>
+        <v>2.917366057767164</v>
       </c>
       <c r="F53">
-        <v>0.8458711785463375</v>
+        <v>0.7860404091118874</v>
       </c>
       <c r="G53">
-        <v>0.0003848337385213725</v>
+        <v>0.0002060584085484883</v>
       </c>
       <c r="H53">
-        <v>1.345195471923256</v>
+        <v>1.376755165514735</v>
       </c>
       <c r="I53">
-        <v>4.660949562945799</v>
+        <v>4.457976950019593</v>
       </c>
     </row>
     <row r="54" spans="1:10">
@@ -4192,19 +4192,19 @@
         <v>76</v>
       </c>
       <c r="E54">
-        <v>-0.6005615618721347</v>
+        <v>-0.5804304890804952</v>
       </c>
       <c r="F54">
-        <v>0.6016704197360456</v>
+        <v>0.6008386784759315</v>
       </c>
       <c r="G54">
-        <v>0.3182032171464896</v>
+        <v>0.3340272537325072</v>
       </c>
       <c r="H54">
-        <v>-1.779813915117882</v>
+        <v>-1.758052659411962</v>
       </c>
       <c r="I54">
-        <v>0.5786907913736121</v>
+        <v>0.5971916812509719</v>
       </c>
     </row>
     <row r="55" spans="1:10">
@@ -4221,19 +4221,19 @@
         <v>77</v>
       </c>
       <c r="E55">
-        <v>0.04841677399052619</v>
+        <v>0.07113471052620553</v>
       </c>
       <c r="F55">
-        <v>0.4502651656788092</v>
+        <v>0.4502752050862395</v>
       </c>
       <c r="G55">
-        <v>0.9143689482931224</v>
+        <v>0.8744721496347461</v>
       </c>
       <c r="H55">
-        <v>-0.8340867342329004</v>
+        <v>-0.8113884745742104</v>
       </c>
       <c r="I55">
-        <v>0.9309202822139526</v>
+        <v>0.9536578956266215</v>
       </c>
     </row>
     <row r="56" spans="1:10">
@@ -4250,19 +4250,19 @@
         <v>78</v>
       </c>
       <c r="E56">
-        <v>-0.5400019663139166</v>
+        <v>-0.4247290354152948</v>
       </c>
       <c r="F56">
-        <v>0.4557867108768484</v>
+        <v>0.4568862373698693</v>
       </c>
       <c r="G56">
-        <v>0.2361087919943252</v>
+        <v>0.3525696239913965</v>
       </c>
       <c r="H56">
-        <v>-1.43332750426451</v>
+        <v>-1.320209605692257</v>
       </c>
       <c r="I56">
-        <v>0.3533235716366767</v>
+        <v>0.4707515348616672</v>
       </c>
     </row>
     <row r="57" spans="1:10">
@@ -4279,19 +4279,19 @@
         <v>79</v>
       </c>
       <c r="E57">
-        <v>-0.3411365833770142</v>
+        <v>-0.2560891021921002</v>
       </c>
       <c r="F57">
-        <v>0.4757606736851447</v>
+        <v>0.4737331237428306</v>
       </c>
       <c r="G57">
-        <v>0.4733531120452293</v>
+        <v>0.588799361676456</v>
       </c>
       <c r="H57">
-        <v>-1.273610369060411</v>
+        <v>-1.184588963011705</v>
       </c>
       <c r="I57">
-        <v>0.5913372023063825</v>
+        <v>0.6724107586275045</v>
       </c>
     </row>
     <row r="58" spans="1:10">
@@ -4308,19 +4308,19 @@
         <v>80</v>
       </c>
       <c r="E58">
-        <v>0.9980516066379581</v>
+        <v>1.087340830812413</v>
       </c>
       <c r="F58">
-        <v>0.4862431074492518</v>
+        <v>0.4913159027988103</v>
       </c>
       <c r="G58">
-        <v>0.04011358259998531</v>
+        <v>0.02688940445398636</v>
       </c>
       <c r="H58">
-        <v>0.04503262830658505</v>
+        <v>0.1243793562949624</v>
       </c>
       <c r="I58">
-        <v>1.951070584969331</v>
+        <v>2.050302305329863</v>
       </c>
     </row>
     <row r="59" spans="1:10">
@@ -4337,19 +4337,19 @@
         <v>81</v>
       </c>
       <c r="E59">
-        <v>1.100079896621413</v>
+        <v>1.101586164410266</v>
       </c>
       <c r="F59">
-        <v>0.7256747071223782</v>
+        <v>0.656070967842712</v>
       </c>
       <c r="G59">
-        <v>0.1295343221918751</v>
+        <v>0.09313926814566875</v>
       </c>
       <c r="H59">
-        <v>-0.3222163938301004</v>
+        <v>-0.1842893038637858</v>
       </c>
       <c r="I59">
-        <v>2.522376187072926</v>
+        <v>2.387461632684317</v>
       </c>
     </row>
     <row r="60" spans="1:10">
@@ -4366,19 +4366,19 @@
         <v>82</v>
       </c>
       <c r="E60">
-        <v>-0.4220676817063762</v>
+        <v>-0.4199375077881112</v>
       </c>
       <c r="F60">
-        <v>0.7280199915416131</v>
+        <v>0.6583701015063103</v>
       </c>
       <c r="G60">
-        <v>0.5620849879766283</v>
+        <v>0.5235751464934311</v>
       </c>
       <c r="H60">
-        <v>-1.848960645153093</v>
+        <v>-1.710319195238459</v>
       </c>
       <c r="I60">
-        <v>1.00482528174034</v>
+        <v>0.8704441796622365</v>
       </c>
     </row>
     <row r="61" spans="1:10">
@@ -4395,19 +4395,19 @@
         <v>83</v>
       </c>
       <c r="E61">
-        <v>-0.2279503124131194</v>
+        <v>-0.214852765769107</v>
       </c>
       <c r="F61">
-        <v>0.721997154554426</v>
+        <v>0.6516104345599983</v>
       </c>
       <c r="G61">
-        <v>0.7522136035838822</v>
+        <v>0.7416071644025184</v>
       </c>
       <c r="H61">
-        <v>-1.643038732280194</v>
+        <v>-1.491985749457198</v>
       </c>
       <c r="I61">
-        <v>1.187138107453955</v>
+        <v>1.062280217918983</v>
       </c>
     </row>
     <row r="62" spans="1:10">
@@ -4424,19 +4424,19 @@
         <v>84</v>
       </c>
       <c r="E62">
-        <v>-0.0313602765105991</v>
+        <v>-0.02012831444562909</v>
       </c>
       <c r="F62">
-        <v>0.7302286689701739</v>
+        <v>0.6609502275066216</v>
       </c>
       <c r="G62">
-        <v>0.9657447151190977</v>
+        <v>0.9757052973157122</v>
       </c>
       <c r="H62">
-        <v>-1.462582168170761</v>
+        <v>-1.315566955932162</v>
       </c>
       <c r="I62">
-        <v>1.399861615149563</v>
+        <v>1.275310327040904</v>
       </c>
     </row>
     <row r="63" spans="1:10">
@@ -4453,19 +4453,19 @@
         <v>85</v>
       </c>
       <c r="E63">
-        <v>0.04767503987344373</v>
+        <v>0.0472923710821806</v>
       </c>
       <c r="F63">
-        <v>0.1108379784868467</v>
+        <v>0.1101391021988578</v>
       </c>
       <c r="G63">
-        <v>0.6670991082894728</v>
+        <v>0.6676411344689668</v>
       </c>
       <c r="H63">
-        <v>-0.1695634060800011</v>
+        <v>-0.1685763025171569</v>
       </c>
       <c r="I63">
-        <v>0.2649134858268886</v>
+        <v>0.2631610446815181</v>
       </c>
     </row>
     <row r="64" spans="1:10">
@@ -4482,22 +4482,22 @@
         <v>92</v>
       </c>
       <c r="E64">
-        <v>0.1322816322484985</v>
+        <v>0.1711235371323078</v>
       </c>
       <c r="F64">
-        <v>0.04824675887388591</v>
+        <v>0.05379442373873606</v>
       </c>
       <c r="G64">
-        <v>0.006110866665473819</v>
+        <v>0.001467349046406702</v>
       </c>
       <c r="H64">
-        <v>0.0377197224848939</v>
+        <v>0.06568840403529858</v>
       </c>
       <c r="I64">
-        <v>0.2268435420121032</v>
+        <v>0.276558670229317</v>
       </c>
       <c r="J64">
-        <v>0.1322816322484985</v>
+        <v>0.1711235371323078</v>
       </c>
     </row>
     <row r="65" spans="1:10">
@@ -4514,22 +4514,22 @@
         <v>87</v>
       </c>
       <c r="E65">
-        <v>0.1548766173827613</v>
+        <v>0.1414189808666478</v>
       </c>
       <c r="F65">
-        <v>0.04527482201395882</v>
+        <v>0.04184791023546278</v>
       </c>
       <c r="G65">
-        <v>0.0006243466323602157</v>
+        <v>0.0007265589414565171</v>
       </c>
       <c r="H65">
-        <v>0.06613959682894086</v>
+        <v>0.0593985839768757</v>
       </c>
       <c r="I65">
-        <v>0.2436136379365818</v>
+        <v>0.22343937775642</v>
       </c>
       <c r="J65">
-        <v>0.1548766173827613</v>
+        <v>0.1414189808666478</v>
       </c>
     </row>
     <row r="66" spans="1:10">
@@ -4546,22 +4546,22 @@
         <v>88</v>
       </c>
       <c r="E66">
-        <v>0.1294911934454973</v>
+        <v>0.1384121531309787</v>
       </c>
       <c r="F66">
-        <v>0.1046191333017976</v>
+        <v>0.1040410668295365</v>
       </c>
       <c r="G66">
-        <v>0.2158128106533763</v>
+        <v>0.1833994355728725</v>
       </c>
       <c r="H66">
-        <v>-0.07555853991982103</v>
+        <v>-0.06550459076803772</v>
       </c>
       <c r="I66">
-        <v>0.3345409268108157</v>
+        <v>0.3423288970299951</v>
       </c>
       <c r="J66">
-        <v>0.1294911934454973</v>
+        <v>0.1384121531309787</v>
       </c>
     </row>
     <row r="67" spans="1:10">
@@ -4578,22 +4578,22 @@
         <v>89</v>
       </c>
       <c r="E67">
-        <v>-0.3597351870777252</v>
+        <v>-0.3547347120513143</v>
       </c>
       <c r="F67">
-        <v>0.07577374024555879</v>
+        <v>0.07603370151289346</v>
       </c>
       <c r="G67">
-        <v>2.05955051475961E-06</v>
+        <v>3.078777828144022E-06</v>
       </c>
       <c r="H67">
-        <v>-0.5082489889329137</v>
+        <v>-0.5037580286278541</v>
       </c>
       <c r="I67">
-        <v>-0.2112213852225368</v>
+        <v>-0.2057113954747745</v>
       </c>
       <c r="J67">
-        <v>-0.3597351870777252</v>
+        <v>-0.3547347120513143</v>
       </c>
     </row>
     <row r="68" spans="1:10">
@@ -4610,22 +4610,22 @@
         <v>90</v>
       </c>
       <c r="E68">
-        <v>0.3005107210120359</v>
+        <v>0.3025847504538222</v>
       </c>
       <c r="F68">
-        <v>0.1067549226957526</v>
+        <v>0.1054669883738317</v>
       </c>
       <c r="G68">
-        <v>0.004878347066047977</v>
+        <v>0.004117722824200883</v>
       </c>
       <c r="H68">
-        <v>0.09127491735600318</v>
+        <v>0.09587325168320746</v>
       </c>
       <c r="I68">
-        <v>0.5097465246680686</v>
+        <v>0.5092962492244369</v>
       </c>
       <c r="J68">
-        <v>0.3005107210120359</v>
+        <v>0.3025847504538222</v>
       </c>
     </row>
     <row r="69" spans="1:10">
@@ -4642,22 +4642,22 @@
         <v>91</v>
       </c>
       <c r="E69">
-        <v>-0.02418750730067423</v>
+        <v>-0.02710320514900285</v>
       </c>
       <c r="F69">
-        <v>0.07407912123337987</v>
+        <v>0.07475877325639842</v>
       </c>
       <c r="G69">
-        <v>0.7440392044310217</v>
+        <v>0.7169469439404681</v>
       </c>
       <c r="H69">
-        <v>-0.1693799169244752</v>
+        <v>-0.1736277082599399</v>
       </c>
       <c r="I69">
-        <v>0.1210049023231267</v>
+        <v>0.1194212979619342</v>
       </c>
       <c r="J69">
-        <v>-0.02418750730067423</v>
+        <v>-0.02710320514900285</v>
       </c>
     </row>
     <row r="70" spans="1:10">
@@ -5069,19 +5069,19 @@
         <v>75</v>
       </c>
       <c r="E83">
-        <v>3.768747692276521</v>
+        <v>4.248478831706663</v>
       </c>
       <c r="F83">
-        <v>9.858411101812312</v>
+        <v>10.83982054634164</v>
       </c>
       <c r="G83">
-        <v>0.7022480984782935</v>
+        <v>0.6951080296905583</v>
       </c>
       <c r="H83">
-        <v>-15.55338301206544</v>
+        <v>-16.99717903800025</v>
       </c>
       <c r="I83">
-        <v>23.09087839661848</v>
+        <v>25.49413670141358</v>
       </c>
     </row>
     <row r="84" spans="1:10">
@@ -5098,19 +5098,19 @@
         <v>80</v>
       </c>
       <c r="E84">
-        <v>2.331458857690044</v>
+        <v>2.243837435745824</v>
       </c>
       <c r="F84">
-        <v>3.353882984654907</v>
+        <v>2.524100167109841</v>
       </c>
       <c r="G84">
-        <v>0.4869599763134116</v>
+        <v>0.3740217346552139</v>
       </c>
       <c r="H84">
-        <v>-4.242031000595276</v>
+        <v>-2.703307985160997</v>
       </c>
       <c r="I84">
-        <v>8.904948715975364</v>
+        <v>7.190982856652644</v>
       </c>
     </row>
     <row r="85" spans="1:10">
@@ -5127,19 +5127,19 @@
         <v>81</v>
       </c>
       <c r="E85">
-        <v>0.9012070061595064</v>
+        <v>0.8138195382517793</v>
       </c>
       <c r="F85">
-        <v>9.851251400021214</v>
+        <v>10.82807355074326</v>
       </c>
       <c r="G85">
-        <v>0.9271100255189695</v>
+        <v>0.9400887668133382</v>
       </c>
       <c r="H85">
-        <v>-18.40689094053186</v>
+        <v>-20.40881464315576</v>
       </c>
       <c r="I85">
-        <v>20.20930495285087</v>
+        <v>22.03645371965931</v>
       </c>
     </row>
     <row r="86" spans="1:10">
@@ -5156,19 +5156,19 @@
         <v>82</v>
       </c>
       <c r="E86">
-        <v>-1.960476632684216</v>
+        <v>-3.155046630895897</v>
       </c>
       <c r="F86">
-        <v>9.964722762465048</v>
+        <v>21.6145318460818</v>
       </c>
       <c r="G86">
-        <v>0.8440296652031867</v>
+        <v>0.8839460421363635</v>
       </c>
       <c r="H86">
-        <v>-21.49097436304218</v>
+        <v>-45.51875059191028</v>
       </c>
       <c r="I86">
-        <v>17.57002109767375</v>
+        <v>39.20865733011848</v>
       </c>
     </row>
     <row r="87" spans="1:10">
@@ -5185,19 +5185,19 @@
         <v>83</v>
       </c>
       <c r="E87">
-        <v>-0.4177201246240076</v>
+        <v>-0.3296787474704433</v>
       </c>
       <c r="F87">
-        <v>9.847845891115433</v>
+        <v>10.82468101015505</v>
       </c>
       <c r="G87">
-        <v>0.9661659490316031</v>
+        <v>0.9757032173010241</v>
       </c>
       <c r="H87">
-        <v>-19.71914339651101</v>
+        <v>-21.54566367150899</v>
       </c>
       <c r="I87">
-        <v>18.883703147263</v>
+        <v>20.88630617656811</v>
       </c>
     </row>
     <row r="88" spans="1:10">
@@ -5214,19 +5214,19 @@
         <v>84</v>
       </c>
       <c r="E88">
-        <v>-0.1937700263819698</v>
+        <v>-0.116995911111562</v>
       </c>
       <c r="F88">
-        <v>9.849491725450276</v>
+        <v>10.82598899805447</v>
       </c>
       <c r="G88">
-        <v>0.9843041504682478</v>
+        <v>0.9913774700716474</v>
       </c>
       <c r="H88">
-        <v>-19.49841907428979</v>
+        <v>-21.33554444432519</v>
       </c>
       <c r="I88">
-        <v>19.11087902152585</v>
+        <v>21.10155262210206</v>
       </c>
     </row>
     <row r="89" spans="1:10">
@@ -5243,19 +5243,19 @@
         <v>85</v>
       </c>
       <c r="E89">
-        <v>-0.1520868063505111</v>
+        <v>-0.1361299221374689</v>
       </c>
       <c r="F89">
-        <v>0.1376814687988474</v>
+        <v>0.1337216547395195</v>
       </c>
       <c r="G89">
-        <v>0.2693208106335139</v>
+        <v>0.3086734156099772</v>
       </c>
       <c r="H89">
-        <v>-0.4219375265348271</v>
+        <v>-0.398219549380027</v>
       </c>
       <c r="I89">
-        <v>0.1177639138338049</v>
+        <v>0.1259597051050891</v>
       </c>
     </row>
     <row r="90" spans="1:10">
@@ -5272,22 +5272,22 @@
         <v>92</v>
       </c>
       <c r="E90">
-        <v>0.9376467025568098</v>
+        <v>1.546515885165592</v>
       </c>
       <c r="F90">
-        <v>0.3683721372607643</v>
+        <v>0.5499977861978362</v>
       </c>
       <c r="G90">
-        <v>0.01091591880427608</v>
+        <v>0.004925618471828861</v>
       </c>
       <c r="H90">
-        <v>0.2156505806176664</v>
+        <v>0.4685400326410722</v>
       </c>
       <c r="I90">
-        <v>1.659642824495953</v>
+        <v>2.624491737690112</v>
       </c>
       <c r="J90">
-        <v>0.9376467025568098</v>
+        <v>1.546515885165592</v>
       </c>
     </row>
     <row r="91" spans="1:10">
@@ -5304,22 +5304,22 @@
         <v>87</v>
       </c>
       <c r="E91">
-        <v>0.2039561605882623</v>
+        <v>0.1442727583266606</v>
       </c>
       <c r="F91">
-        <v>0.1108020597310869</v>
+        <v>0.1021174793657897</v>
       </c>
       <c r="G91">
-        <v>0.0656618165557489</v>
+        <v>0.157711129716964</v>
       </c>
       <c r="H91">
-        <v>-0.0132118858975239</v>
+        <v>-0.05587382342229941</v>
       </c>
       <c r="I91">
-        <v>0.4211242070740485</v>
+        <v>0.3444193400756206</v>
       </c>
       <c r="J91">
-        <v>0.2039561605882623</v>
+        <v>0.1442727583266606</v>
       </c>
     </row>
     <row r="92" spans="1:10">
@@ -5336,22 +5336,22 @@
         <v>88</v>
       </c>
       <c r="E92">
-        <v>0.007212615504369017</v>
+        <v>0.05084352044059733</v>
       </c>
       <c r="F92">
-        <v>0.2526590322802555</v>
+        <v>0.2491638513080231</v>
       </c>
       <c r="G92">
-        <v>0.9772260149409779</v>
+        <v>0.8383092936623524</v>
       </c>
       <c r="H92">
-        <v>-0.4879899881336748</v>
+        <v>-0.4375086543724213</v>
       </c>
       <c r="I92">
-        <v>0.5024152191424128</v>
+        <v>0.5391956952536159</v>
       </c>
       <c r="J92">
-        <v>0.007212615504369017</v>
+        <v>0.05084352044059733</v>
       </c>
     </row>
     <row r="93" spans="1:10">
@@ -5368,22 +5368,22 @@
         <v>89</v>
       </c>
       <c r="E93">
-        <v>-1.084539152377894</v>
+        <v>-1.056605498875292</v>
       </c>
       <c r="F93">
-        <v>0.4095347608645611</v>
+        <v>0.4030533154527287</v>
       </c>
       <c r="G93">
-        <v>0.008091625911413106</v>
+        <v>0.008754297701142593</v>
       </c>
       <c r="H93">
-        <v>-1.887212534089657</v>
+        <v>-1.846575481012102</v>
       </c>
       <c r="I93">
-        <v>-0.2818657706661304</v>
+        <v>-0.2666355167384827</v>
       </c>
       <c r="J93">
-        <v>-1.084539152377894</v>
+        <v>-1.056605498875292</v>
       </c>
     </row>
     <row r="94" spans="1:10">
@@ -5400,22 +5400,22 @@
         <v>90</v>
       </c>
       <c r="E94">
-        <v>0.7812553935753863</v>
+        <v>0.7333888968278429</v>
       </c>
       <c r="F94">
-        <v>0.3077800323877884</v>
+        <v>0.3102800945842114</v>
       </c>
       <c r="G94">
-        <v>0.01113745213170189</v>
+        <v>0.01809663115522448</v>
       </c>
       <c r="H94">
-        <v>0.1780176149347495</v>
+        <v>0.1252510863231072</v>
       </c>
       <c r="I94">
-        <v>1.384493172216023</v>
+        <v>1.341526707332579</v>
       </c>
       <c r="J94">
-        <v>0.7812553935753863</v>
+        <v>0.7333888968278429</v>
       </c>
     </row>
     <row r="95" spans="1:10">
@@ -5432,22 +5432,22 @@
         <v>91</v>
       </c>
       <c r="E95">
-        <v>0.09042056682961208</v>
+        <v>0.06751518199563347</v>
       </c>
       <c r="F95">
-        <v>0.2141185223125586</v>
+        <v>0.2074492045303057</v>
       </c>
       <c r="G95">
-        <v>0.6728118019428135</v>
+        <v>0.7448374605320107</v>
       </c>
       <c r="H95">
-        <v>-0.3292440253259387</v>
+        <v>-0.3390777875052492</v>
       </c>
       <c r="I95">
-        <v>0.5100851589851628</v>
+        <v>0.4741081514965162</v>
       </c>
       <c r="J95">
-        <v>0.09042056682961208</v>
+        <v>0.06751518199563347</v>
       </c>
     </row>
     <row r="96" spans="1:10">
@@ -5979,13 +5979,13 @@
         <v>1142</v>
       </c>
       <c r="E3">
-        <v>3674.110604186647</v>
+        <v>3673.043584197633</v>
       </c>
       <c r="F3">
-        <v>3759.799722820318</v>
+        <v>3758.732702831304</v>
       </c>
       <c r="G3">
-        <v>0.23027942674959</v>
+        <v>0.230998274092541</v>
       </c>
       <c r="I3" t="s">
         <v>66</v>
@@ -6562,19 +6562,19 @@
         <v>75</v>
       </c>
       <c r="E19">
-        <v>3.003072517434528</v>
+        <v>2.917366057767164</v>
       </c>
       <c r="F19">
-        <v>0.8458711785463375</v>
+        <v>0.7860404091118874</v>
       </c>
       <c r="G19">
-        <v>0.0003848337385213725</v>
+        <v>0.0002060584085484883</v>
       </c>
       <c r="H19">
-        <v>1.345195471923256</v>
+        <v>1.376755165514735</v>
       </c>
       <c r="I19">
-        <v>4.660949562945799</v>
+        <v>4.457976950019593</v>
       </c>
     </row>
     <row r="20" spans="1:10">
@@ -6591,19 +6591,19 @@
         <v>76</v>
       </c>
       <c r="E20">
-        <v>-0.6005615618721347</v>
+        <v>-0.5804304890804952</v>
       </c>
       <c r="F20">
-        <v>0.6016704197360456</v>
+        <v>0.6008386784759315</v>
       </c>
       <c r="G20">
-        <v>0.3182032171464896</v>
+        <v>0.3340272537325072</v>
       </c>
       <c r="H20">
-        <v>-1.779813915117882</v>
+        <v>-1.758052659411962</v>
       </c>
       <c r="I20">
-        <v>0.5786907913736121</v>
+        <v>0.5971916812509719</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -6620,19 +6620,19 @@
         <v>77</v>
       </c>
       <c r="E21">
-        <v>0.04841677399052619</v>
+        <v>0.07113471052620553</v>
       </c>
       <c r="F21">
-        <v>0.4502651656788092</v>
+        <v>0.4502752050862395</v>
       </c>
       <c r="G21">
-        <v>0.9143689482931224</v>
+        <v>0.8744721496347461</v>
       </c>
       <c r="H21">
-        <v>-0.8340867342329004</v>
+        <v>-0.8113884745742104</v>
       </c>
       <c r="I21">
-        <v>0.9309202822139526</v>
+        <v>0.9536578956266215</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -6649,19 +6649,19 @@
         <v>78</v>
       </c>
       <c r="E22">
-        <v>-0.5400019663139166</v>
+        <v>-0.4247290354152948</v>
       </c>
       <c r="F22">
-        <v>0.4557867108768484</v>
+        <v>0.4568862373698693</v>
       </c>
       <c r="G22">
-        <v>0.2361087919943252</v>
+        <v>0.3525696239913965</v>
       </c>
       <c r="H22">
-        <v>-1.43332750426451</v>
+        <v>-1.320209605692257</v>
       </c>
       <c r="I22">
-        <v>0.3533235716366767</v>
+        <v>0.4707515348616672</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -6678,19 +6678,19 @@
         <v>79</v>
       </c>
       <c r="E23">
-        <v>-0.3411365833770142</v>
+        <v>-0.2560891021921002</v>
       </c>
       <c r="F23">
-        <v>0.4757606736851447</v>
+        <v>0.4737331237428306</v>
       </c>
       <c r="G23">
-        <v>0.4733531120452293</v>
+        <v>0.588799361676456</v>
       </c>
       <c r="H23">
-        <v>-1.273610369060411</v>
+        <v>-1.184588963011705</v>
       </c>
       <c r="I23">
-        <v>0.5913372023063825</v>
+        <v>0.6724107586275045</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -6707,19 +6707,19 @@
         <v>80</v>
       </c>
       <c r="E24">
-        <v>0.9980516066379581</v>
+        <v>1.087340830812413</v>
       </c>
       <c r="F24">
-        <v>0.4862431074492518</v>
+        <v>0.4913159027988103</v>
       </c>
       <c r="G24">
-        <v>0.04011358259998531</v>
+        <v>0.02688940445398636</v>
       </c>
       <c r="H24">
-        <v>0.04503262830658505</v>
+        <v>0.1243793562949624</v>
       </c>
       <c r="I24">
-        <v>1.951070584969331</v>
+        <v>2.050302305329863</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -6736,19 +6736,19 @@
         <v>81</v>
       </c>
       <c r="E25">
-        <v>1.100079896621413</v>
+        <v>1.101586164410266</v>
       </c>
       <c r="F25">
-        <v>0.7256747071223782</v>
+        <v>0.656070967842712</v>
       </c>
       <c r="G25">
-        <v>0.1295343221918751</v>
+        <v>0.09313926814566875</v>
       </c>
       <c r="H25">
-        <v>-0.3222163938301004</v>
+        <v>-0.1842893038637858</v>
       </c>
       <c r="I25">
-        <v>2.522376187072926</v>
+        <v>2.387461632684317</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -6765,19 +6765,19 @@
         <v>82</v>
       </c>
       <c r="E26">
-        <v>-0.4220676817063762</v>
+        <v>-0.4199375077881112</v>
       </c>
       <c r="F26">
-        <v>0.7280199915416131</v>
+        <v>0.6583701015063103</v>
       </c>
       <c r="G26">
-        <v>0.5620849879766283</v>
+        <v>0.5235751464934311</v>
       </c>
       <c r="H26">
-        <v>-1.848960645153093</v>
+        <v>-1.710319195238459</v>
       </c>
       <c r="I26">
-        <v>1.00482528174034</v>
+        <v>0.8704441796622365</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -6794,19 +6794,19 @@
         <v>83</v>
       </c>
       <c r="E27">
-        <v>-0.2279503124131194</v>
+        <v>-0.214852765769107</v>
       </c>
       <c r="F27">
-        <v>0.721997154554426</v>
+        <v>0.6516104345599983</v>
       </c>
       <c r="G27">
-        <v>0.7522136035838822</v>
+        <v>0.7416071644025184</v>
       </c>
       <c r="H27">
-        <v>-1.643038732280194</v>
+        <v>-1.491985749457198</v>
       </c>
       <c r="I27">
-        <v>1.187138107453955</v>
+        <v>1.062280217918983</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -6823,19 +6823,19 @@
         <v>84</v>
       </c>
       <c r="E28">
-        <v>-0.0313602765105991</v>
+        <v>-0.02012831444562909</v>
       </c>
       <c r="F28">
-        <v>0.7302286689701739</v>
+        <v>0.6609502275066216</v>
       </c>
       <c r="G28">
-        <v>0.9657447151190977</v>
+        <v>0.9757052973157122</v>
       </c>
       <c r="H28">
-        <v>-1.462582168170761</v>
+        <v>-1.315566955932162</v>
       </c>
       <c r="I28">
-        <v>1.399861615149563</v>
+        <v>1.275310327040904</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -6852,19 +6852,19 @@
         <v>85</v>
       </c>
       <c r="E29">
-        <v>0.04767503987344373</v>
+        <v>0.0472923710821806</v>
       </c>
       <c r="F29">
-        <v>0.1108379784868467</v>
+        <v>0.1101391021988578</v>
       </c>
       <c r="G29">
-        <v>0.6670991082894728</v>
+        <v>0.6676411344689668</v>
       </c>
       <c r="H29">
-        <v>-0.1695634060800011</v>
+        <v>-0.1685763025171569</v>
       </c>
       <c r="I29">
-        <v>0.2649134858268886</v>
+        <v>0.2631610446815181</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -6881,22 +6881,22 @@
         <v>92</v>
       </c>
       <c r="E30">
-        <v>0.1322816322484985</v>
+        <v>0.1711235371323078</v>
       </c>
       <c r="F30">
-        <v>0.04824675887388591</v>
+        <v>0.05379442373873606</v>
       </c>
       <c r="G30">
-        <v>0.006110866665473819</v>
+        <v>0.001467349046406702</v>
       </c>
       <c r="H30">
-        <v>0.0377197224848939</v>
+        <v>0.06568840403529858</v>
       </c>
       <c r="I30">
-        <v>0.2268435420121032</v>
+        <v>0.276558670229317</v>
       </c>
       <c r="J30">
-        <v>0.1322816322484985</v>
+        <v>0.1711235371323078</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -6913,22 +6913,22 @@
         <v>87</v>
       </c>
       <c r="E31">
-        <v>0.1548766173827613</v>
+        <v>0.1414189808666478</v>
       </c>
       <c r="F31">
-        <v>0.04527482201395882</v>
+        <v>0.04184791023546278</v>
       </c>
       <c r="G31">
-        <v>0.0006243466323602157</v>
+        <v>0.0007265589414565171</v>
       </c>
       <c r="H31">
-        <v>0.06613959682894086</v>
+        <v>0.0593985839768757</v>
       </c>
       <c r="I31">
-        <v>0.2436136379365818</v>
+        <v>0.22343937775642</v>
       </c>
       <c r="J31">
-        <v>0.1548766173827613</v>
+        <v>0.1414189808666478</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -6945,22 +6945,22 @@
         <v>88</v>
       </c>
       <c r="E32">
-        <v>0.1294911934454973</v>
+        <v>0.1384121531309787</v>
       </c>
       <c r="F32">
-        <v>0.1046191333017976</v>
+        <v>0.1040410668295365</v>
       </c>
       <c r="G32">
-        <v>0.2158128106533763</v>
+        <v>0.1833994355728725</v>
       </c>
       <c r="H32">
-        <v>-0.07555853991982103</v>
+        <v>-0.06550459076803772</v>
       </c>
       <c r="I32">
-        <v>0.3345409268108157</v>
+        <v>0.3423288970299951</v>
       </c>
       <c r="J32">
-        <v>0.1294911934454973</v>
+        <v>0.1384121531309787</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -6977,22 +6977,22 @@
         <v>89</v>
       </c>
       <c r="E33">
-        <v>-0.3597351870777252</v>
+        <v>-0.3547347120513143</v>
       </c>
       <c r="F33">
-        <v>0.07577374024555879</v>
+        <v>0.07603370151289346</v>
       </c>
       <c r="G33">
-        <v>2.05955051475961E-06</v>
+        <v>3.078777828144022E-06</v>
       </c>
       <c r="H33">
-        <v>-0.5082489889329137</v>
+        <v>-0.5037580286278541</v>
       </c>
       <c r="I33">
-        <v>-0.2112213852225368</v>
+        <v>-0.2057113954747745</v>
       </c>
       <c r="J33">
-        <v>-0.3597351870777252</v>
+        <v>-0.3547347120513143</v>
       </c>
     </row>
     <row r="34" spans="1:10">
@@ -7009,22 +7009,22 @@
         <v>90</v>
       </c>
       <c r="E34">
-        <v>0.3005107210120359</v>
+        <v>0.3025847504538222</v>
       </c>
       <c r="F34">
-        <v>0.1067549226957526</v>
+        <v>0.1054669883738317</v>
       </c>
       <c r="G34">
-        <v>0.004878347066047977</v>
+        <v>0.004117722824200883</v>
       </c>
       <c r="H34">
-        <v>0.09127491735600318</v>
+        <v>0.09587325168320746</v>
       </c>
       <c r="I34">
-        <v>0.5097465246680686</v>
+        <v>0.5092962492244369</v>
       </c>
       <c r="J34">
-        <v>0.3005107210120359</v>
+        <v>0.3025847504538222</v>
       </c>
     </row>
     <row r="35" spans="1:10">
@@ -7041,22 +7041,22 @@
         <v>91</v>
       </c>
       <c r="E35">
-        <v>-0.02418750730067423</v>
+        <v>-0.02710320514900285</v>
       </c>
       <c r="F35">
-        <v>0.07407912123337987</v>
+        <v>0.07475877325639842</v>
       </c>
       <c r="G35">
-        <v>0.7440392044310217</v>
+        <v>0.7169469439404681</v>
       </c>
       <c r="H35">
-        <v>-0.1693799169244752</v>
+        <v>-0.1736277082599399</v>
       </c>
       <c r="I35">
-        <v>0.1210049023231267</v>
+        <v>0.1194212979619342</v>
       </c>
       <c r="J35">
-        <v>-0.02418750730067423</v>
+        <v>-0.02710320514900285</v>
       </c>
     </row>
   </sheetData>
@@ -7141,13 +7141,13 @@
         <v>126</v>
       </c>
       <c r="E3">
-        <v>262.4070276459344</v>
+        <v>260.5765054617245</v>
       </c>
       <c r="F3">
-        <v>299.2786924363036</v>
+        <v>297.4481702520937</v>
       </c>
       <c r="G3">
-        <v>0.3002978010149173</v>
+        <v>0.3103895584745069</v>
       </c>
       <c r="I3" t="s">
         <v>66</v>

</xml_diff>